<commit_message>
Expand regional API catalog and update schema
</commit_message>
<xml_diff>
--- a/job_api_catalog.xlsx
+++ b/job_api_catalog.xlsx
@@ -8194,7 +8194,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>Not Recommended</t>
+          <t>No Public API</t>
         </is>
       </c>
     </row>
@@ -8271,7 +8271,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>Not Recommended</t>
+          <t>No Public API</t>
         </is>
       </c>
     </row>
@@ -8348,7 +8348,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>Not Recommended</t>
+          <t>No Public API</t>
         </is>
       </c>
     </row>
@@ -8425,7 +8425,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>Not Recommended</t>
+          <t>Enterprise Only</t>
         </is>
       </c>
     </row>
@@ -8502,7 +8502,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>Not Recommended</t>
+          <t>Enterprise Only</t>
         </is>
       </c>
     </row>
@@ -8964,7 +8964,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>Not Recommended</t>
+          <t>Enterprise Only</t>
         </is>
       </c>
     </row>
@@ -9041,7 +9041,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>Not Recommended</t>
+          <t>Enterprise Only</t>
         </is>
       </c>
     </row>
@@ -9118,7 +9118,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>Not Recommended</t>
+          <t>Enterprise Only</t>
         </is>
       </c>
     </row>
@@ -9195,7 +9195,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>Not Recommended</t>
+          <t>No Public API</t>
         </is>
       </c>
     </row>
@@ -9272,7 +9272,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>Not Recommended</t>
+          <t>No Public API</t>
         </is>
       </c>
     </row>
@@ -9868,7 +9868,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Whether this (API, Region) row is Integrated (live in jobs.py today), Recommended (researched, not yet integrated, report recommends adding), or Not Recommended (researched and explicitly ruled out - e.g. no public API, partner-only, or per-tenant-only).</t>
+          <t>Whether this (API, Region) row is Integrated (live in jobs.py today), Recommended (researched, not yet integrated, report recommends adding), Not Recommended (researched and the report explicitly advises against pursuing it - e.g. scraping-only with a stated legal/maintenance caution), No Public API (no official or workable public endpoint exists at all), or Enterprise Only (an API exists but only via a paid/partner/per-tenant enterprise agreement, not a public aggregatable feed).</t>
         </is>
       </c>
     </row>

</xml_diff>